<commit_message>
Add explicit join spec for differently-named source columns
- load_source_frame accepts `file@acc_col=file_col` — joins an added
  source where the shared-column auto-join cannot apply
  (e.g. transform_lab,region_ref@country=ctry)
- auto-join error now tells the user the explicit syntax exists
- ER-125 exercises the path live; region_ref.csv is the demo fixture
- 3 new unit tests (join, bad column, no-shared-column hint)

Generated with [Devin](https://devin.ai)

Co-Authored-By: Devin <158243242+devin-ai-integration[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/rules/migration_rules.xlsx
+++ b/data/rules/migration_rules.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L34"/>
+  <dimension ref="A1:L35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2222,6 +2222,60 @@
         </is>
       </c>
       <c r="L34" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>ER-125</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>transform_lab,region_ref@country=ctry</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>country</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>transform_lab</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>region</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>LOOKUP</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>lookup(region)</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>lab_id</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
         <is>
           <t>yes</t>
         </is>

</xml_diff>